<commit_message>
ingesta: snapshot 2026-10-13 18:07 UTC
</commit_message>
<xml_diff>
--- a/data_lake/acumulado_tempmax_mes/dt=2026-10-13/Temp-max-octubre-26.xlsx
+++ b/data_lake/acumulado_tempmax_mes/dt=2026-10-13/Temp-max-octubre-26.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\Mi unidad\OSPA\02. Datos Diarios\Tablas\Datos hidrometeorologicos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F71B1EDC-3F54-41FE-85DA-A98DF4C85251}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F7EA488-74E4-47CA-ACAA-2CD60BA7ACFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="355" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9459,7 +9459,9 @@
       <c r="O5" s="63">
         <v>31.7</v>
       </c>
-      <c r="P5" s="63"/>
+      <c r="P5" s="63">
+        <v>31.9</v>
+      </c>
       <c r="Q5" s="63"/>
       <c r="R5" s="63"/>
       <c r="S5" s="63"/>
@@ -9481,7 +9483,7 @@
       <c r="AI5" s="63"/>
       <c r="AJ5" s="36">
         <f>+IF(SUM($E5:$AI5)&gt;0,LOOKUP(1000,$E5:$AI5),NA())</f>
-        <v>31.7</v>
+        <v>31.9</v>
       </c>
       <c r="AK5" s="21">
         <f>+MAX($E5:$AI5)</f>
@@ -9553,7 +9555,9 @@
       <c r="O6" s="63">
         <v>31.1</v>
       </c>
-      <c r="P6" s="63"/>
+      <c r="P6" s="63">
+        <v>31.7</v>
+      </c>
       <c r="Q6" s="63"/>
       <c r="R6" s="63"/>
       <c r="S6" s="63"/>
@@ -9575,7 +9579,7 @@
       <c r="AI6" s="63"/>
       <c r="AJ6" s="36">
         <f t="shared" ref="AJ6:AJ48" si="0">+IF(SUM($E6:$AI6)&gt;0,LOOKUP(1000,$E6:$AI6),NA())</f>
-        <v>31.1</v>
+        <v>31.7</v>
       </c>
       <c r="AK6" s="21">
         <f t="shared" ref="AK6:AK48" si="1">+MAX($E6:$AI6)</f>
@@ -9647,7 +9651,9 @@
       <c r="O7" s="63">
         <v>35.200000000000003</v>
       </c>
-      <c r="P7" s="63"/>
+      <c r="P7" s="63">
+        <v>34.799999999999997</v>
+      </c>
       <c r="Q7" s="63"/>
       <c r="R7" s="63"/>
       <c r="S7" s="63"/>
@@ -9669,7 +9675,7 @@
       <c r="AI7" s="63"/>
       <c r="AJ7" s="36">
         <f t="shared" si="0"/>
-        <v>35.200000000000003</v>
+        <v>34.799999999999997</v>
       </c>
       <c r="AK7" s="21">
         <f t="shared" si="1"/>
@@ -9741,7 +9747,9 @@
       <c r="O8" s="63">
         <v>34.1</v>
       </c>
-      <c r="P8" s="63"/>
+      <c r="P8" s="63">
+        <v>33.9</v>
+      </c>
       <c r="Q8" s="63"/>
       <c r="R8" s="63"/>
       <c r="S8" s="63"/>
@@ -9763,7 +9771,7 @@
       <c r="AI8" s="63"/>
       <c r="AJ8" s="36">
         <f t="shared" si="0"/>
-        <v>34.1</v>
+        <v>33.9</v>
       </c>
       <c r="AK8" s="21">
         <f t="shared" si="1"/>
@@ -9835,7 +9843,9 @@
       <c r="O9" s="63">
         <v>36.299999999999997</v>
       </c>
-      <c r="P9" s="63"/>
+      <c r="P9" s="63">
+        <v>34.4</v>
+      </c>
       <c r="Q9" s="63"/>
       <c r="R9" s="63"/>
       <c r="S9" s="63"/>
@@ -9857,7 +9867,7 @@
       <c r="AI9" s="63"/>
       <c r="AJ9" s="36">
         <f t="shared" si="0"/>
-        <v>36.299999999999997</v>
+        <v>34.4</v>
       </c>
       <c r="AK9" s="21">
         <f t="shared" si="1"/>
@@ -9929,7 +9939,9 @@
       <c r="O10" s="63">
         <v>34.5</v>
       </c>
-      <c r="P10" s="63"/>
+      <c r="P10" s="63">
+        <v>32.9</v>
+      </c>
       <c r="Q10" s="63"/>
       <c r="R10" s="63"/>
       <c r="S10" s="63"/>
@@ -9951,7 +9963,7 @@
       <c r="AI10" s="63"/>
       <c r="AJ10" s="36">
         <f t="shared" si="0"/>
-        <v>34.5</v>
+        <v>32.9</v>
       </c>
       <c r="AK10" s="21">
         <f t="shared" si="1"/>
@@ -10023,7 +10035,9 @@
       <c r="O11" s="63">
         <v>35.6</v>
       </c>
-      <c r="P11" s="63"/>
+      <c r="P11" s="63">
+        <v>32.799999999999997</v>
+      </c>
       <c r="Q11" s="63"/>
       <c r="R11" s="63"/>
       <c r="S11" s="63"/>
@@ -10045,7 +10059,7 @@
       <c r="AI11" s="63"/>
       <c r="AJ11" s="36">
         <f t="shared" si="0"/>
-        <v>35.6</v>
+        <v>32.799999999999997</v>
       </c>
       <c r="AK11" s="21">
         <f t="shared" si="1"/>
@@ -10117,7 +10131,9 @@
       <c r="O12" s="63">
         <v>33.799999999999997</v>
       </c>
-      <c r="P12" s="63"/>
+      <c r="P12" s="63">
+        <v>31.4</v>
+      </c>
       <c r="Q12" s="63"/>
       <c r="R12" s="63"/>
       <c r="S12" s="63"/>
@@ -10139,7 +10155,7 @@
       <c r="AI12" s="63"/>
       <c r="AJ12" s="36">
         <f t="shared" si="0"/>
-        <v>33.799999999999997</v>
+        <v>31.4</v>
       </c>
       <c r="AK12" s="21">
         <f t="shared" si="1"/>
@@ -10211,7 +10227,9 @@
       <c r="O13" s="63">
         <v>34.799999999999997</v>
       </c>
-      <c r="P13" s="63"/>
+      <c r="P13" s="63">
+        <v>32</v>
+      </c>
       <c r="Q13" s="63"/>
       <c r="R13" s="63"/>
       <c r="S13" s="63"/>
@@ -10233,7 +10251,7 @@
       <c r="AI13" s="63"/>
       <c r="AJ13" s="36">
         <f t="shared" si="0"/>
-        <v>34.799999999999997</v>
+        <v>32</v>
       </c>
       <c r="AK13" s="21">
         <f t="shared" si="1"/>
@@ -10305,7 +10323,9 @@
       <c r="O14" s="63">
         <v>34.1</v>
       </c>
-      <c r="P14" s="63"/>
+      <c r="P14" s="63">
+        <v>32.700000000000003</v>
+      </c>
       <c r="Q14" s="63"/>
       <c r="R14" s="63"/>
       <c r="S14" s="63"/>
@@ -10327,7 +10347,7 @@
       <c r="AI14" s="63"/>
       <c r="AJ14" s="36">
         <f t="shared" si="0"/>
-        <v>34.1</v>
+        <v>32.700000000000003</v>
       </c>
       <c r="AK14" s="21">
         <f t="shared" si="1"/>
@@ -10399,7 +10419,9 @@
       <c r="O15" s="63">
         <v>32.6</v>
       </c>
-      <c r="P15" s="63"/>
+      <c r="P15" s="63">
+        <v>29.3</v>
+      </c>
       <c r="Q15" s="63"/>
       <c r="R15" s="63"/>
       <c r="S15" s="63"/>
@@ -10421,7 +10443,7 @@
       <c r="AI15" s="63"/>
       <c r="AJ15" s="36">
         <f t="shared" si="0"/>
-        <v>32.6</v>
+        <v>29.3</v>
       </c>
       <c r="AK15" s="21">
         <f t="shared" si="1"/>
@@ -10542,7 +10564,9 @@
       <c r="O17" s="63">
         <v>34.6</v>
       </c>
-      <c r="P17" s="63"/>
+      <c r="P17" s="63">
+        <v>27.4</v>
+      </c>
       <c r="Q17" s="63"/>
       <c r="R17" s="63"/>
       <c r="S17" s="63"/>
@@ -10564,7 +10588,7 @@
       <c r="AI17" s="63"/>
       <c r="AJ17" s="36">
         <f t="shared" si="0"/>
-        <v>34.6</v>
+        <v>27.4</v>
       </c>
       <c r="AK17" s="21">
         <f t="shared" si="1"/>
@@ -10636,7 +10660,9 @@
       <c r="O18" s="63">
         <v>29</v>
       </c>
-      <c r="P18" s="63"/>
+      <c r="P18" s="63">
+        <v>25.1</v>
+      </c>
       <c r="Q18" s="63"/>
       <c r="R18" s="63"/>
       <c r="S18" s="63"/>
@@ -10658,7 +10684,7 @@
       <c r="AI18" s="63"/>
       <c r="AJ18" s="36">
         <f t="shared" si="0"/>
-        <v>29</v>
+        <v>25.1</v>
       </c>
       <c r="AK18" s="21">
         <f t="shared" si="1"/>
@@ -10730,7 +10756,9 @@
       <c r="O19" s="63">
         <v>35.1</v>
       </c>
-      <c r="P19" s="63"/>
+      <c r="P19" s="63">
+        <v>32.4</v>
+      </c>
       <c r="Q19" s="63"/>
       <c r="R19" s="63"/>
       <c r="S19" s="63"/>
@@ -10752,7 +10780,7 @@
       <c r="AI19" s="63"/>
       <c r="AJ19" s="36">
         <f t="shared" si="0"/>
-        <v>35.1</v>
+        <v>32.4</v>
       </c>
       <c r="AK19" s="21">
         <f t="shared" si="1"/>
@@ -10824,7 +10852,9 @@
       <c r="O20" s="63">
         <v>28.8</v>
       </c>
-      <c r="P20" s="63"/>
+      <c r="P20" s="63">
+        <v>22.6</v>
+      </c>
       <c r="Q20" s="63"/>
       <c r="R20" s="63"/>
       <c r="S20" s="63"/>
@@ -10846,7 +10876,7 @@
       <c r="AI20" s="63"/>
       <c r="AJ20" s="36">
         <f t="shared" si="0"/>
-        <v>28.8</v>
+        <v>22.6</v>
       </c>
       <c r="AK20" s="21">
         <f t="shared" si="1"/>
@@ -10918,7 +10948,9 @@
       <c r="O21" s="63">
         <v>23.6</v>
       </c>
-      <c r="P21" s="63"/>
+      <c r="P21" s="63">
+        <v>18.600000000000001</v>
+      </c>
       <c r="Q21" s="63"/>
       <c r="R21" s="63"/>
       <c r="S21" s="63"/>
@@ -10940,7 +10972,7 @@
       <c r="AI21" s="63"/>
       <c r="AJ21" s="36">
         <f t="shared" si="0"/>
-        <v>23.6</v>
+        <v>18.600000000000001</v>
       </c>
       <c r="AK21" s="21">
         <f t="shared" si="1"/>
@@ -11078,7 +11110,9 @@
       <c r="O23" s="63">
         <v>27.9</v>
       </c>
-      <c r="P23" s="63"/>
+      <c r="P23" s="63">
+        <v>24.8</v>
+      </c>
       <c r="Q23" s="63"/>
       <c r="R23" s="63"/>
       <c r="S23" s="63"/>
@@ -11100,7 +11134,7 @@
       <c r="AI23" s="63"/>
       <c r="AJ23" s="36">
         <f t="shared" si="0"/>
-        <v>27.9</v>
+        <v>24.8</v>
       </c>
       <c r="AK23" s="21">
         <f t="shared" si="1"/>
@@ -11172,7 +11206,9 @@
       <c r="O24" s="63">
         <v>27.8</v>
       </c>
-      <c r="P24" s="63"/>
+      <c r="P24" s="63">
+        <v>24.7</v>
+      </c>
       <c r="Q24" s="63"/>
       <c r="R24" s="63"/>
       <c r="S24" s="63"/>
@@ -11194,7 +11230,7 @@
       <c r="AI24" s="63"/>
       <c r="AJ24" s="36">
         <f t="shared" si="0"/>
-        <v>27.8</v>
+        <v>24.7</v>
       </c>
       <c r="AK24" s="21">
         <f t="shared" si="1"/>
@@ -11266,7 +11302,9 @@
       <c r="O25" s="63">
         <v>30.7</v>
       </c>
-      <c r="P25" s="63"/>
+      <c r="P25" s="63">
+        <v>26</v>
+      </c>
       <c r="Q25" s="63"/>
       <c r="R25" s="63"/>
       <c r="S25" s="63"/>
@@ -11288,7 +11326,7 @@
       <c r="AI25" s="63"/>
       <c r="AJ25" s="36">
         <f t="shared" si="0"/>
-        <v>30.7</v>
+        <v>26</v>
       </c>
       <c r="AK25" s="21">
         <f t="shared" si="1"/>
@@ -11360,7 +11398,9 @@
       <c r="O26" s="63">
         <v>20.3</v>
       </c>
-      <c r="P26" s="63"/>
+      <c r="P26" s="63">
+        <v>18</v>
+      </c>
       <c r="Q26" s="63"/>
       <c r="R26" s="63"/>
       <c r="S26" s="63"/>
@@ -11382,7 +11422,7 @@
       <c r="AI26" s="63"/>
       <c r="AJ26" s="36">
         <f t="shared" si="0"/>
-        <v>20.3</v>
+        <v>18</v>
       </c>
       <c r="AK26" s="21">
         <f t="shared" si="1"/>
@@ -11454,7 +11494,9 @@
       <c r="O27" s="63">
         <v>22.2</v>
       </c>
-      <c r="P27" s="63"/>
+      <c r="P27" s="63">
+        <v>21</v>
+      </c>
       <c r="Q27" s="63"/>
       <c r="R27" s="63"/>
       <c r="S27" s="63"/>
@@ -11476,7 +11518,7 @@
       <c r="AI27" s="63"/>
       <c r="AJ27" s="36">
         <f t="shared" si="0"/>
-        <v>22.2</v>
+        <v>21</v>
       </c>
       <c r="AK27" s="21">
         <f t="shared" si="1"/>
@@ -11548,7 +11590,9 @@
       <c r="O28" s="63">
         <v>30.1</v>
       </c>
-      <c r="P28" s="63"/>
+      <c r="P28" s="63">
+        <v>27.3</v>
+      </c>
       <c r="Q28" s="63"/>
       <c r="R28" s="63"/>
       <c r="S28" s="63"/>
@@ -11570,7 +11614,7 @@
       <c r="AI28" s="63"/>
       <c r="AJ28" s="36">
         <f t="shared" si="0"/>
-        <v>30.1</v>
+        <v>27.3</v>
       </c>
       <c r="AK28" s="21">
         <f t="shared" si="1"/>
@@ -11706,7 +11750,9 @@
       <c r="O30" s="63">
         <v>36.200000000000003</v>
       </c>
-      <c r="P30" s="63"/>
+      <c r="P30" s="63">
+        <v>34.799999999999997</v>
+      </c>
       <c r="Q30" s="63"/>
       <c r="R30" s="63"/>
       <c r="S30" s="63"/>
@@ -11728,7 +11774,7 @@
       <c r="AI30" s="63"/>
       <c r="AJ30" s="36">
         <f t="shared" si="0"/>
-        <v>36.200000000000003</v>
+        <v>34.799999999999997</v>
       </c>
       <c r="AK30" s="21">
         <f t="shared" si="1"/>
@@ -11800,7 +11846,9 @@
       <c r="O31" s="63">
         <v>25.2</v>
       </c>
-      <c r="P31" s="63"/>
+      <c r="P31" s="63">
+        <v>22.6</v>
+      </c>
       <c r="Q31" s="63"/>
       <c r="R31" s="63"/>
       <c r="S31" s="63"/>
@@ -11822,7 +11870,7 @@
       <c r="AI31" s="63"/>
       <c r="AJ31" s="36">
         <f t="shared" si="0"/>
-        <v>25.2</v>
+        <v>22.6</v>
       </c>
       <c r="AK31" s="21">
         <f t="shared" si="1"/>
@@ -11894,7 +11942,9 @@
       <c r="O32" s="63">
         <v>19.8</v>
       </c>
-      <c r="P32" s="63"/>
+      <c r="P32" s="63">
+        <v>18.8</v>
+      </c>
       <c r="Q32" s="63"/>
       <c r="R32" s="63"/>
       <c r="S32" s="63"/>
@@ -11916,7 +11966,7 @@
       <c r="AI32" s="63"/>
       <c r="AJ32" s="36">
         <f t="shared" si="0"/>
-        <v>19.8</v>
+        <v>18.8</v>
       </c>
       <c r="AK32" s="21">
         <f t="shared" si="1"/>
@@ -11988,7 +12038,9 @@
       <c r="O33" s="63">
         <v>17</v>
       </c>
-      <c r="P33" s="63"/>
+      <c r="P33" s="63">
+        <v>17.600000000000001</v>
+      </c>
       <c r="Q33" s="63"/>
       <c r="R33" s="63"/>
       <c r="S33" s="63"/>
@@ -12010,7 +12062,7 @@
       <c r="AI33" s="63"/>
       <c r="AJ33" s="36">
         <f t="shared" si="0"/>
-        <v>17</v>
+        <v>17.600000000000001</v>
       </c>
       <c r="AK33" s="21">
         <f t="shared" si="1"/>
@@ -12134,7 +12186,9 @@
       <c r="O35" s="63">
         <v>30.2</v>
       </c>
-      <c r="P35" s="63"/>
+      <c r="P35" s="63">
+        <v>28.2</v>
+      </c>
       <c r="Q35" s="63"/>
       <c r="R35" s="63"/>
       <c r="S35" s="63"/>
@@ -12156,7 +12210,7 @@
       <c r="AI35" s="63"/>
       <c r="AJ35" s="36">
         <f t="shared" si="0"/>
-        <v>30.2</v>
+        <v>28.2</v>
       </c>
       <c r="AK35" s="21">
         <f t="shared" si="1"/>
@@ -12347,7 +12401,9 @@
       <c r="O38" s="63">
         <v>30.7</v>
       </c>
-      <c r="P38" s="63"/>
+      <c r="P38" s="63">
+        <v>32.9</v>
+      </c>
       <c r="Q38" s="63"/>
       <c r="R38" s="63"/>
       <c r="S38" s="63"/>
@@ -12369,7 +12425,7 @@
       <c r="AI38" s="63"/>
       <c r="AJ38" s="36">
         <f t="shared" si="0"/>
-        <v>30.7</v>
+        <v>32.9</v>
       </c>
       <c r="AK38" s="21">
         <f t="shared" si="1"/>
@@ -12442,7 +12498,9 @@
       <c r="O39" s="63">
         <v>33.799999999999997</v>
       </c>
-      <c r="P39" s="63"/>
+      <c r="P39" s="63">
+        <v>32.799999999999997</v>
+      </c>
       <c r="Q39" s="63"/>
       <c r="R39" s="63"/>
       <c r="S39" s="63"/>
@@ -12464,7 +12522,7 @@
       <c r="AI39" s="63"/>
       <c r="AJ39" s="36">
         <f t="shared" si="0"/>
-        <v>33.799999999999997</v>
+        <v>32.799999999999997</v>
       </c>
       <c r="AK39" s="21">
         <f t="shared" si="1"/>
@@ -12537,7 +12595,9 @@
       <c r="O40" s="63">
         <v>31.7</v>
       </c>
-      <c r="P40" s="63"/>
+      <c r="P40" s="63">
+        <v>29.7</v>
+      </c>
       <c r="Q40" s="63"/>
       <c r="R40" s="63"/>
       <c r="S40" s="63"/>
@@ -12559,7 +12619,7 @@
       <c r="AI40" s="63"/>
       <c r="AJ40" s="36">
         <f t="shared" si="0"/>
-        <v>31.7</v>
+        <v>29.7</v>
       </c>
       <c r="AK40" s="21">
         <f t="shared" si="1"/>
@@ -12791,7 +12851,9 @@
       <c r="O43" s="63">
         <v>31.4</v>
       </c>
-      <c r="P43" s="63"/>
+      <c r="P43" s="63">
+        <v>33.6</v>
+      </c>
       <c r="Q43" s="63"/>
       <c r="R43" s="63"/>
       <c r="S43" s="63"/>
@@ -12813,7 +12875,7 @@
       <c r="AI43" s="63"/>
       <c r="AJ43" s="36">
         <f t="shared" si="0"/>
-        <v>31.4</v>
+        <v>33.6</v>
       </c>
       <c r="AK43" s="21">
         <f t="shared" si="1"/>
@@ -12886,7 +12948,9 @@
       <c r="O44" s="29">
         <v>34</v>
       </c>
-      <c r="P44" s="29"/>
+      <c r="P44" s="29">
+        <v>31.3</v>
+      </c>
       <c r="Q44" s="29"/>
       <c r="R44" s="29"/>
       <c r="S44" s="29"/>
@@ -12908,7 +12972,7 @@
       <c r="AI44" s="63"/>
       <c r="AJ44" s="36">
         <f t="shared" si="0"/>
-        <v>34</v>
+        <v>31.3</v>
       </c>
       <c r="AK44" s="21">
         <f t="shared" si="1"/>
@@ -12981,7 +13045,9 @@
       <c r="O45" s="63">
         <v>34</v>
       </c>
-      <c r="P45" s="63"/>
+      <c r="P45" s="63">
+        <v>32</v>
+      </c>
       <c r="Q45" s="63"/>
       <c r="R45" s="63"/>
       <c r="S45" s="63"/>
@@ -13003,7 +13069,7 @@
       <c r="AI45" s="63"/>
       <c r="AJ45" s="36">
         <f t="shared" si="0"/>
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="AK45" s="21">
         <f t="shared" si="1"/>
@@ -13208,7 +13274,9 @@
       <c r="O48" s="63">
         <v>34.1</v>
       </c>
-      <c r="P48" s="63"/>
+      <c r="P48" s="63">
+        <v>34.200000000000003</v>
+      </c>
       <c r="Q48" s="63"/>
       <c r="R48" s="63"/>
       <c r="S48" s="63"/>
@@ -13230,7 +13298,7 @@
       <c r="AI48" s="63"/>
       <c r="AJ48" s="36">
         <f t="shared" si="0"/>
-        <v>34.1</v>
+        <v>34.200000000000003</v>
       </c>
       <c r="AK48" s="21">
         <f t="shared" si="1"/>
@@ -26308,12 +26376,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="E1:E2"/>
     <mergeCell ref="M1:M2"/>
     <mergeCell ref="N1:N2"/>
     <mergeCell ref="O1:O2"/>
@@ -26323,6 +26385,12 @@
     <mergeCell ref="J1:J2"/>
     <mergeCell ref="K1:K2"/>
     <mergeCell ref="L1:L2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="E1:E2"/>
   </mergeCells>
   <conditionalFormatting sqref="D4:O13 D15:O31 D33:O34 D36:O46">
     <cfRule type="cellIs" dxfId="0" priority="1" stopIfTrue="1" operator="equal">

</xml_diff>